<commit_message>
feat(store): 行内编辑设备 family + Excel 状态下拉
- 门店搭建页设备行删除按钮左侧加"编辑"铅笔, 打开抽屉编辑底层
  Equipment(family); 保存后所有引用该设备的行联动更新 + router.refresh。
  EquipmentForm 加 embedded 模式复用; 新增 EquipmentEditDrawer。
- Excel 加"状态(下拉选择)"列(New/Existing/(E)Relocate/Remove 数据校验), 加宽。
- tsc=0, eslint=0, 门店页冒烟 200 正常。

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/设备规格表-待处理清单.xlsx
+++ b/docs/设备规格表-待处理清单.xlsx
@@ -44,7 +44,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +69,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,6 +129,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -491,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -499,10 +507,11 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="46" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -565,6 +574,11 @@
           <t>备注（手填）</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>状态（下拉选择）</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -606,6 +620,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="11" t="n"/>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -647,6 +662,7 @@
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="11" t="n"/>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -685,6 +701,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="11" t="n"/>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -723,6 +740,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="11" t="n"/>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -760,6 +778,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
+      <c r="J9" s="11" t="n"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -797,6 +816,7 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="11" t="n"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="4" t="n">
@@ -838,6 +858,7 @@
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="11" t="n"/>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="4" t="n">
@@ -875,6 +896,7 @@
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="11" t="n"/>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="4" t="n">
@@ -912,6 +934,7 @@
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="11" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -949,6 +972,7 @@
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="11" t="n"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="4" t="n">
@@ -990,6 +1014,7 @@
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="11" t="n"/>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="4" t="n">
@@ -1031,6 +1056,7 @@
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="11" t="n"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="4" t="n">
@@ -1068,6 +1094,7 @@
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="11" t="n"/>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -1105,6 +1132,7 @@
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="11" t="n"/>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -1142,6 +1170,7 @@
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="11" t="n"/>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="4" t="n">
@@ -1183,6 +1212,7 @@
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="11" t="n"/>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="4" t="n">
@@ -1224,6 +1254,7 @@
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="11" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="4" t="n">
@@ -1261,6 +1292,7 @@
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="11" t="n"/>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="4" t="n">
@@ -1302,6 +1334,7 @@
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="11" t="n"/>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="4" t="n">
@@ -1343,6 +1376,7 @@
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="11" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="4" t="n">
@@ -1372,6 +1406,7 @@
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="11" t="n"/>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="A26" s="4" t="n">
@@ -1413,6 +1448,7 @@
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="11" t="n"/>
     </row>
     <row r="27" ht="46" customHeight="1">
       <c r="A27" s="4" t="n">
@@ -1454,6 +1490,7 @@
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr"/>
+      <c r="J27" s="11" t="n"/>
     </row>
     <row r="28" ht="46" customHeight="1">
       <c r="A28" s="4" t="n">
@@ -1495,6 +1532,7 @@
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="11" t="n"/>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="A29" s="4" t="n">
@@ -1536,6 +1574,7 @@
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr"/>
+      <c r="J29" s="11" t="n"/>
     </row>
     <row r="30" ht="46" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -1577,6 +1616,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="11" t="n"/>
     </row>
     <row r="31" ht="46" customHeight="1">
       <c r="A31" s="4" t="n">
@@ -1614,6 +1654,7 @@
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr"/>
+      <c r="J31" s="11" t="n"/>
     </row>
     <row r="32" ht="46" customHeight="1">
       <c r="A32" s="4" t="n">
@@ -1651,6 +1692,7 @@
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="11" t="n"/>
     </row>
     <row r="33" ht="46" customHeight="1">
       <c r="A33" s="4" t="n">
@@ -1692,6 +1734,7 @@
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
+      <c r="J33" s="11" t="n"/>
     </row>
     <row r="34" ht="46" customHeight="1">
       <c r="A34" s="4" t="n">
@@ -1729,6 +1772,7 @@
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="11" t="n"/>
     </row>
     <row r="35" ht="46" customHeight="1">
       <c r="A35" s="4" t="n">
@@ -1766,6 +1810,7 @@
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
+      <c r="J35" s="11" t="n"/>
     </row>
     <row r="36" ht="46" customHeight="1">
       <c r="A36" s="4" t="n">
@@ -1803,6 +1848,7 @@
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="11" t="n"/>
     </row>
     <row r="37" ht="46" customHeight="1">
       <c r="A37" s="4" t="n">
@@ -1840,6 +1886,7 @@
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr"/>
+      <c r="J37" s="11" t="n"/>
     </row>
     <row r="38" ht="46" customHeight="1">
       <c r="A38" s="4" t="n">
@@ -1877,6 +1924,7 @@
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="11" t="n"/>
     </row>
     <row r="39" ht="46" customHeight="1">
       <c r="A39" s="4" t="n">
@@ -1914,6 +1962,7 @@
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="11" t="n"/>
     </row>
     <row r="40" ht="46" customHeight="1">
       <c r="A40" s="4" t="n">
@@ -1951,6 +2000,7 @@
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="11" t="n"/>
     </row>
     <row r="41" ht="46" customHeight="1">
       <c r="A41" s="4" t="n">
@@ -1988,6 +2038,7 @@
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="11" t="n"/>
     </row>
     <row r="42" ht="46" customHeight="1">
       <c r="A42" s="4" t="n">
@@ -2025,6 +2076,7 @@
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr"/>
+      <c r="J42" s="11" t="n"/>
     </row>
     <row r="43" ht="46" customHeight="1">
       <c r="A43" s="4" t="n">
@@ -2062,6 +2114,7 @@
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="11" t="n"/>
     </row>
     <row r="44" ht="46" customHeight="1">
       <c r="A44" s="4" t="n">
@@ -2099,6 +2152,7 @@
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="11" t="n"/>
     </row>
     <row r="45" ht="46" customHeight="1">
       <c r="A45" s="4" t="n">
@@ -2136,6 +2190,7 @@
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="11" t="n"/>
     </row>
     <row r="46" ht="46" customHeight="1">
       <c r="A46" s="4" t="n">
@@ -2173,6 +2228,7 @@
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="11" t="n"/>
     </row>
     <row r="47" ht="46" customHeight="1">
       <c r="A47" s="4" t="n">
@@ -2210,6 +2266,7 @@
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr"/>
+      <c r="J47" s="11" t="n"/>
     </row>
     <row r="48" ht="46" customHeight="1">
       <c r="A48" s="4" t="n">
@@ -2247,6 +2304,7 @@
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="11" t="n"/>
     </row>
     <row r="49" ht="46" customHeight="1">
       <c r="A49" s="4" t="n">
@@ -2284,12 +2342,18 @@
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="J5:J49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="设备状态" prompt="点单元格右侧箭头选择" type="list">
+      <formula1>"New,Existing,(E)Relocate,Remove"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2300,15 +2364,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F213"/>
+  <dimension ref="A1:G213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2356,6 +2421,11 @@
           <t>规格表文件 / 线索</t>
         </is>
       </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>状态（下拉选择）</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -2386,6 +2456,7 @@
           <t>001_Dell-POS System_OptiPlex GX260.pdf</t>
         </is>
       </c>
+      <c r="G5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -2416,6 +2487,7 @@
           <t>002_Toledo-Scan Weigh Scale.pdf</t>
         </is>
       </c>
+      <c r="G6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -2446,6 +2518,7 @@
           <t>003_BIZERBA KHII -datasheet_kh_ii_100_en.pdf</t>
         </is>
       </c>
+      <c r="G7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -2468,6 +2541,7 @@
           <t>004_Toledo-Self Service Scale_UC-CWT EVO.pdf</t>
         </is>
       </c>
+      <c r="G8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -2490,6 +2564,7 @@
           <t>005_Mettler Toledo-Floor Scale_2158 Vertex.pdf</t>
         </is>
       </c>
+      <c r="G9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -2520,6 +2595,7 @@
           <t>006_Lottery Machine.pdf</t>
         </is>
       </c>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -2550,6 +2626,7 @@
           <t>007 55inch Floor standing digital signage.pdf</t>
         </is>
       </c>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -2580,6 +2657,7 @@
           <t>008_Kronos-InTouch 9100 Badge Terminal.pdf</t>
         </is>
       </c>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2610,6 +2688,7 @@
           <t>009_Turn-O-Matic-Number System-S3.pdf</t>
         </is>
       </c>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -2640,6 +2719,7 @@
           <t>010_Samsung-LED Menu Board_H5003.pdf</t>
         </is>
       </c>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -2670,6 +2750,7 @@
           <t>011 Produce Dry Table.pdf</t>
         </is>
       </c>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -2700,6 +2781,7 @@
           <t>012 Superstructure Madix TL-Series.pdf</t>
         </is>
       </c>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -2730,6 +2812,7 @@
           <t>013 Produce Bin.pdf</t>
         </is>
       </c>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -2752,6 +2835,7 @@
           <t>014_Trade Fixtures-Bulk Display_RMT-14001B.pdf</t>
         </is>
       </c>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -2782,6 +2866,7 @@
           <t>015 Madix Grocery Gondola 016 Grocery Gondola End.pdf</t>
         </is>
       </c>
+      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -2812,6 +2897,7 @@
           <t>015 Madix Grocery Gondola 016 Grocery Gondola End.pdf</t>
         </is>
       </c>
+      <c r="G20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -2842,6 +2928,7 @@
           <t>017_Grocery Rice Display.pdf</t>
         </is>
       </c>
+      <c r="G21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -2872,6 +2959,7 @@
           <t>018_Ivar-Check Stand End-Display.pdf</t>
         </is>
       </c>
+      <c r="G22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -2902,6 +2990,7 @@
           <t>019_Sonozaire_model_overview_v1.pdf</t>
         </is>
       </c>
+      <c r="G23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -2932,6 +3021,7 @@
           <t>020_Marathon-Baler_V6030HD.pdf</t>
         </is>
       </c>
+      <c r="G24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2962,6 +3052,7 @@
           <t>021_Marathon-Trash Compactor_RJ-250SC.pdf</t>
         </is>
       </c>
+      <c r="G25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -2992,6 +3083,7 @@
           <t>021_Marathon-Trash Compactor_RJ-250SC.pdf</t>
         </is>
       </c>
+      <c r="G26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -3022,6 +3114,7 @@
           <t>022_Mars-Air Curtain.pdf</t>
         </is>
       </c>
+      <c r="G27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -3052,6 +3145,7 @@
           <t>023 Manual Pallet Jacks.pdf</t>
         </is>
       </c>
+      <c r="G28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -3082,6 +3176,7 @@
           <t>024 Electric Pallet Jack.pdf</t>
         </is>
       </c>
+      <c r="G29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -3112,6 +3207,7 @@
           <t>025 Walkie Straddle.pdf</t>
         </is>
       </c>
+      <c r="G30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -3134,6 +3230,7 @@
           <t>027_Alvarado-Post Guard.pdf</t>
         </is>
       </c>
+      <c r="G31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -3164,6 +3261,7 @@
           <t>028_Self checkout_Toshiba Cashless 2 Bag 6800.pdf</t>
         </is>
       </c>
+      <c r="G32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -3194,6 +3292,7 @@
           <t>030_Killion_Check-Stand_KCu3500.pdf</t>
         </is>
       </c>
+      <c r="G33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3220,6 +3319,7 @@
           <t>030_Killion_Single Check-Stand_KCu3500 P4348RM SCAN AND PASS.pdf</t>
         </is>
       </c>
+      <c r="G34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -3250,6 +3350,7 @@
           <t>031_Custom_Customer Service Counter.pdf</t>
         </is>
       </c>
+      <c r="G35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3280,6 +3381,7 @@
           <t>033_Custom-Trash Receptacle.pdf</t>
         </is>
       </c>
+      <c r="G36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3310,6 +3412,7 @@
           <t>033_Trash Receptacle - Single.pdf</t>
         </is>
       </c>
+      <c r="G37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -3340,6 +3443,7 @@
           <t>033_Trash Receptacle - Double.pdf</t>
         </is>
       </c>
+      <c r="G38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -3370,6 +3474,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -3400,6 +3505,7 @@
           <t>035 Bakery Back Counter.pdf</t>
         </is>
       </c>
+      <c r="G40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -3430,6 +3536,7 @@
           <t>1OVe3IZV35fLAw3MT7v2oMPl-bK2gU0jC.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -3460,6 +3567,7 @@
           <t>037_Bakery Toast Rack Spec.pdf</t>
         </is>
       </c>
+      <c r="G42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -3490,6 +3598,7 @@
           <t>038_Custom-Condiments Counter.pdf</t>
         </is>
       </c>
+      <c r="G43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -3520,6 +3629,7 @@
           <t>039 Hatco FDWD-2X.PDF</t>
         </is>
       </c>
+      <c r="G44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -3550,6 +3660,7 @@
           <t>040 Antunes SDC-500.pdf</t>
         </is>
       </c>
+      <c r="G45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -3580,6 +3691,7 @@
           <t>041 HATCO-GR2SDH-36D.pdf</t>
         </is>
       </c>
+      <c r="G46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -3610,6 +3722,7 @@
           <t>042_Custom Hot Deli SS Front Service Counter.pdf</t>
         </is>
       </c>
+      <c r="G47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -3640,6 +3753,7 @@
           <t>043_Custom Hot Deli SS Back Counter.pdf</t>
         </is>
       </c>
+      <c r="G48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -3666,6 +3780,7 @@
           <t>044_Misc Bakery Display_Marco_3tierTabel.pdf</t>
         </is>
       </c>
+      <c r="G49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -3696,6 +3811,7 @@
           <t>045_Bakery Tray Tong Station Spec (new style).pdf</t>
         </is>
       </c>
+      <c r="G50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -3726,6 +3842,7 @@
           <t>048-048A_Traulsen-Reach-In Refrigerator G Series.pdf</t>
         </is>
       </c>
+      <c r="G51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -3756,6 +3873,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -3786,6 +3904,7 @@
           <t>050_Hill Phoenix Produce wall case O5DM.pdf</t>
         </is>
       </c>
+      <c r="G53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -3816,6 +3935,7 @@
           <t>052_Hill Phoenix produce island- OIP OIPB.pdf</t>
         </is>
       </c>
+      <c r="G54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -3847,6 +3967,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -3878,6 +3999,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -3908,6 +4030,7 @@
           <t>053 Deli-Dairy Open Multideck - 5DMLH-NRG-diplay-case-tech-reference-sheet-6.0..pdf</t>
         </is>
       </c>
+      <c r="G57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -3938,6 +4061,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -3968,6 +4092,7 @@
           <t>054 Deli-Dairy Closed Multideck VRB-display-case-tech-reference-sheet-6.1.pdf</t>
         </is>
       </c>
+      <c r="G59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -3998,6 +4123,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -4028,6 +4154,7 @@
           <t>055_Hill Phoenix - multi deck Meat - Seafood open cs O5M.pdf</t>
         </is>
       </c>
+      <c r="G61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n">
@@ -4058,6 +4185,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -4088,6 +4216,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -4118,6 +4247,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -4148,6 +4278,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -4178,6 +4309,7 @@
           <t>058_Hill Phoenix -Frozen reach in case-VNRZ.pdf</t>
         </is>
       </c>
+      <c r="G66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -4208,6 +4340,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n">
@@ -4238,6 +4371,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -4268,6 +4402,7 @@
           <t>060_AHT_PARIS R290_2015.pdf</t>
         </is>
       </c>
+      <c r="G69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -4294,6 +4429,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -4324,6 +4460,7 @@
           <t>060 Excellence Island Cases HR-18H HR-21H.pdf</t>
         </is>
       </c>
+      <c r="G71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n">
@@ -4354,6 +4491,7 @@
           <t>068_Turbo Air-Self Service Cake Display Case_TOM-75LBSF.pdf</t>
         </is>
       </c>
+      <c r="G72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -4384,6 +4522,7 @@
           <t>056_Hill Phoenix Seafood Service case -SSAM-RG.pdf</t>
         </is>
       </c>
+      <c r="G73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n">
@@ -4414,6 +4553,7 @@
           <t>063_Hill Phoenix Meat Service Case SGM-display-case-tech-reference-sheet-v2.pdf</t>
         </is>
       </c>
+      <c r="G74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -4444,6 +4584,7 @@
           <t>064_Hill Phoenix Bakery Service BLF.pdf</t>
         </is>
       </c>
+      <c r="G75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n">
@@ -4474,6 +4615,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -4504,6 +4646,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -4534,6 +4677,7 @@
           <t>074_Beverage-Air-Underconter Refrigerator_UCR27.pdf</t>
         </is>
       </c>
+      <c r="G78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -4564,6 +4708,7 @@
           <t>068_Turbo Air-Self Service Cake Display Case_TOM-75LBSF.pdf</t>
         </is>
       </c>
+      <c r="G79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n">
@@ -4594,6 +4739,7 @@
           <t>069_Turbo Air-Self Service Cake Display Case_TOM-40LBSF.pdf</t>
         </is>
       </c>
+      <c r="G80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -4624,6 +4770,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -4654,6 +4801,7 @@
           <t>071_Heatcraft-Air Cooled Condenser.pdf</t>
         </is>
       </c>
+      <c r="G82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -4684,6 +4832,7 @@
           <t>072-073_Hill Phoenix_Walk-In Cooler+Freezer.pdf</t>
         </is>
       </c>
+      <c r="G83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n">
@@ -4714,6 +4863,7 @@
           <t>072-073_Hill Phoenix_Walk-In Cooler+Freezer.pdf</t>
         </is>
       </c>
+      <c r="G84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -4744,6 +4894,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n">
@@ -4774,6 +4925,7 @@
           <t>076-077_Traulsen-Reach-In Refrigerator G Series.pdf</t>
         </is>
       </c>
+      <c r="G86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
@@ -4804,6 +4956,7 @@
           <t>076-077_Traulsen-Reach-In Refrigerator G Series.pdf</t>
         </is>
       </c>
+      <c r="G87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n">
@@ -4834,6 +4987,7 @@
           <t>078-079_Traulsen-Reach-In Freezer G Series.pdf</t>
         </is>
       </c>
+      <c r="G88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -4864,6 +5018,7 @@
           <t>078-079_Traulsen-Reach-In Freezer G Series.pdf</t>
         </is>
       </c>
+      <c r="G89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
@@ -4894,6 +5049,7 @@
           <t>080_TRUE-Flat Top Cold Table TUC-60 TWT-60.pdf</t>
         </is>
       </c>
+      <c r="G90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
@@ -4924,6 +5080,7 @@
           <t>081A True TSSU-60-16-HC.SpecSheet.pdf</t>
         </is>
       </c>
+      <c r="G91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n">
@@ -4954,6 +5111,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
@@ -4984,6 +5142,7 @@
           <t>083_Frigidaire-Refrigerator_FFTR1814Q.pdf</t>
         </is>
       </c>
+      <c r="G93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n">
@@ -5014,6 +5173,7 @@
           <t>085_Kloppenberg-Ice Storage Bin_2115.pdf</t>
         </is>
       </c>
+      <c r="G94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -5044,6 +5204,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n">
@@ -5074,6 +5235,7 @@
           <t>087 Ice-O-Matic MFI1256A.SpecSheet.pdf</t>
         </is>
       </c>
+      <c r="G96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n">
@@ -5104,6 +5266,7 @@
           <t>088_Ice-O-Matic-Cube Ice Maker_ICEU300-305.pdf</t>
         </is>
       </c>
+      <c r="G97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n">
@@ -5134,6 +5297,7 @@
           <t>089 Ice-O-Matic B110PS.SpecShee.pdf</t>
         </is>
       </c>
+      <c r="G98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -5164,6 +5328,7 @@
           <t>090_Advance Tabco-Wall Mount Hand Sink_7-PS-66.pdf</t>
         </is>
       </c>
+      <c r="G99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n">
@@ -5194,6 +5359,7 @@
           <t>15EFeYnumFnxaNMsPpKR8uJSLMjocLgHu.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n">
@@ -5224,6 +5390,7 @@
           <t>091_Trough Sink_ELRF82000-ELRF-82000.pdf</t>
         </is>
       </c>
+      <c r="G101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n">
@@ -5254,6 +5421,7 @@
           <t>092_Kohler-Bathroom SS Undermount Sink_K-2602.pdf</t>
         </is>
       </c>
+      <c r="G102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n">
@@ -5284,6 +5452,7 @@
           <t>093 SLOAN Trough Sink Faucet EAF-100.pdf</t>
         </is>
       </c>
+      <c r="G103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n">
@@ -5314,6 +5483,7 @@
           <t>094_Aero_1Comp-Sink-1DB_MF1-2418-18R.pdf</t>
         </is>
       </c>
+      <c r="G104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n">
@@ -5344,6 +5514,7 @@
           <t>094B_Aero_1Comp-Sink-1DB_MF1-2418-18L.pdf</t>
         </is>
       </c>
+      <c r="G105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n">
@@ -5374,6 +5545,7 @@
           <t>095-096_Aero-2Comp Sink 2DB_MF2-24XX-XXLR.pdf</t>
         </is>
       </c>
+      <c r="G106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n">
@@ -5404,6 +5576,7 @@
           <t>095-096_Aero-2Comp Sink 2DB_MF2-24XX-18LR.pdf</t>
         </is>
       </c>
+      <c r="G107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n">
@@ -5434,6 +5607,7 @@
           <t>097-098_Aero-3Comp Sink 2DB_MF3-24XX-XXLR.pdf</t>
         </is>
       </c>
+      <c r="G108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n">
@@ -5464,6 +5638,7 @@
           <t>097-098_Aero-3Comp Sink 2DB_MF3-24XX-XXLR.pdf</t>
         </is>
       </c>
+      <c r="G109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n">
@@ -5494,6 +5669,7 @@
           <t>100_Advance Tabco-Mop Sink_9-OP-28.pdf</t>
         </is>
       </c>
+      <c r="G110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n">
@@ -5524,6 +5700,7 @@
           <t>1UIQHIQn9DpELmAfGJ-5Pciibo0YKSFxL.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G111" s="11" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n">
@@ -5554,6 +5731,7 @@
           <t>101_Fisher-Mop Sink Faucet_8261.pdf</t>
         </is>
       </c>
+      <c r="G112" s="11" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n">
@@ -5584,6 +5762,7 @@
           <t>102_Fisher-Wok Range Faucet_60224.pdf</t>
         </is>
       </c>
+      <c r="G113" s="11" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n">
@@ -5614,6 +5793,7 @@
           <t>103_Moen-Commercial Lav Faucet_M-Bition.pdf</t>
         </is>
       </c>
+      <c r="G114" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n">
@@ -5644,6 +5824,7 @@
           <t>104_Fisher-Kitchen Faucet_60143.pdf</t>
         </is>
       </c>
+      <c r="G115" s="11" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n">
@@ -5674,6 +5855,7 @@
           <t>105_Rheem-Ruud_Water-Heater_G100-200A.pdf</t>
         </is>
       </c>
+      <c r="G116" s="11" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n">
@@ -5704,6 +5886,7 @@
           <t>106_Halsey-Taylor_Contour-Bi-Lev-Drink-Fountain.pdf</t>
         </is>
       </c>
+      <c r="G117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n">
@@ -5734,6 +5917,7 @@
           <t>106B_Elkay_LZSTL8WSLP.pdf</t>
         </is>
       </c>
+      <c r="G118" s="11" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n">
@@ -5764,6 +5948,7 @@
           <t>107_Krowne-Drop-In Beverage Sink_HS-1419.pdf</t>
         </is>
       </c>
+      <c r="G119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n">
@@ -5794,6 +5979,7 @@
           <t>108_Xlerator Hand-Dryer.pdf</t>
         </is>
       </c>
+      <c r="G120" s="11" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n">
@@ -5824,6 +6010,7 @@
           <t>110_ISS_Gold-Bond-Wire-Shelf_P74NY.pdf</t>
         </is>
       </c>
+      <c r="G121" s="11" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n">
@@ -5854,6 +6041,7 @@
           <t>111 Trough Sink Soap Dispenser SLOAN ESD-1500-CP.pdf</t>
         </is>
       </c>
+      <c r="G122" s="11" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n">
@@ -5884,6 +6072,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G123" s="11" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n">
@@ -5914,6 +6103,7 @@
           <t>114_Employee Lockers GSW 2DR 5DR.pdf</t>
         </is>
       </c>
+      <c r="G124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n">
@@ -5936,6 +6126,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G125" s="11" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n">
@@ -5966,6 +6157,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G126" s="11" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n">
@@ -5996,6 +6188,7 @@
           <t>119_Advance Tabco-Mop Rack_K242.pdf</t>
         </is>
       </c>
+      <c r="G127" s="11" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n">
@@ -6026,6 +6219,7 @@
           <t>120_Eagle Group-Stainless Steel Work Table_T3060SB.pdf</t>
         </is>
       </c>
+      <c r="G128" s="11" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n">
@@ -6056,6 +6250,7 @@
           <t>121 Eagle Group - Poly Top Table CT3060S.pdf</t>
         </is>
       </c>
+      <c r="G129" s="11" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n">
@@ -6086,6 +6281,7 @@
           <t>122_SCALEMATE_Wrapper.pdf</t>
         </is>
       </c>
+      <c r="G130" s="11" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n">
@@ -6116,6 +6312,7 @@
           <t>123_Eagle Group-Equipment Stand_MS3024.pdf</t>
         </is>
       </c>
+      <c r="G131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n">
@@ -6146,6 +6343,7 @@
           <t>124_Custom_ADA Counter.pdf</t>
         </is>
       </c>
+      <c r="G132" s="11" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n">
@@ -6176,6 +6374,7 @@
           <t>125_Hobart-Meat Saw_6801.pdf</t>
         </is>
       </c>
+      <c r="G133" s="11" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n">
@@ -6206,6 +6405,7 @@
           <t>126_Hobart-Meat Grinder_4146.pdf</t>
         </is>
       </c>
+      <c r="G134" s="11" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n">
@@ -6236,6 +6436,7 @@
           <t>127A Tabletop Meat Slicer - Bizerba - GSP-HD.pdf</t>
         </is>
       </c>
+      <c r="G135" s="11" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n">
@@ -6266,6 +6467,7 @@
           <t>127 Tabletop Meat Slicer - Hobart - HS7N.pdf</t>
         </is>
       </c>
+      <c r="G136" s="11" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n">
@@ -6296,6 +6498,7 @@
           <t>128_Biro-Meat Tenderlicer_Pro-9.pdf</t>
         </is>
       </c>
+      <c r="G137" s="11" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n">
@@ -6326,6 +6529,7 @@
           <t>129_Biro auto meat slicer 109pc.pdf</t>
         </is>
       </c>
+      <c r="G138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n">
@@ -6356,6 +6560,7 @@
           <t>130 Seafood Steamer Groen SSB-5G.SpecSheet.pdf</t>
         </is>
       </c>
+      <c r="G139" s="11" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n">
@@ -6386,6 +6591,7 @@
           <t>131A Self Contained Bi-Level Fish Tank 5FT.pdf</t>
         </is>
       </c>
+      <c r="G140" s="11" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n">
@@ -6416,6 +6622,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G141" s="11" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n">
@@ -6446,6 +6653,7 @@
           <t>132_Self Contained Seafood Tank 4FT.pdf</t>
         </is>
       </c>
+      <c r="G142" s="11" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n">
@@ -6476,6 +6684,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n">
@@ -6506,6 +6715,7 @@
           <t>134L_General-Equip_Fish-Cutting-Table-L.pdf</t>
         </is>
       </c>
+      <c r="G144" s="11" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n">
@@ -6536,6 +6746,7 @@
           <t>134R_General-Equip_Fish-Cutting-Table-R.pdf</t>
         </is>
       </c>
+      <c r="G145" s="11" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n">
@@ -6566,6 +6777,7 @@
           <t>137_Cambro-Ice Caddy_ICS125L.pdf</t>
         </is>
       </c>
+      <c r="G146" s="11" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n">
@@ -6596,6 +6808,7 @@
           <t>139A Seafood Ice Display.pdf</t>
         </is>
       </c>
+      <c r="G147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n">
@@ -6626,6 +6839,7 @@
           <t>140_CaptiveAire-Type-I Exhaust Hood Wall_ND-2.pdf</t>
         </is>
       </c>
+      <c r="G148" s="11" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n">
@@ -6656,6 +6870,7 @@
           <t>141_CaptiveAire-Type-II Exhaust Hood Wall_VHB.pdf</t>
         </is>
       </c>
+      <c r="G149" s="11" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n">
@@ -6686,6 +6901,7 @@
           <t>149-149A-150-151-152_Imperial-Chinese Wok Range-1-8 Holes.pdf</t>
         </is>
       </c>
+      <c r="G150" s="11" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n">
@@ -6716,6 +6932,7 @@
           <t>145_General Equip-BBQ Oven_GNR4848.pdf</t>
         </is>
       </c>
+      <c r="G151" s="11" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n">
@@ -6746,6 +6963,7 @@
           <t>145 BBQ Oven CMP_202_G.pdf</t>
         </is>
       </c>
+      <c r="G152" s="11" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n">
@@ -6776,6 +6994,7 @@
           <t>146-147_American Range-HD-Stock-Pot-Stoves_ARSP18.pdf</t>
         </is>
       </c>
+      <c r="G153" s="11" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n">
@@ -6806,6 +7025,7 @@
           <t>148_Deep Fryer-Pitco Solstice Gas-SG18.pdf</t>
         </is>
       </c>
+      <c r="G154" s="11" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n">
@@ -6836,6 +7056,7 @@
           <t>L006 Deep Fryer ATFS-50.pdf</t>
         </is>
       </c>
+      <c r="G155" s="11" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n">
@@ -6866,6 +7087,7 @@
           <t>149-149A-150-151-152_Imperial-Chinese Wok Range-1-8 Holes.pdf</t>
         </is>
       </c>
+      <c r="G156" s="11" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n">
@@ -6896,6 +7118,7 @@
           <t>149 B &amp; 150B_ACE Wok range (2 burner &amp; 3 burners).pdf</t>
         </is>
       </c>
+      <c r="G157" s="11" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n">
@@ -6926,6 +7149,7 @@
           <t>149-149A-150-151-152_Imperial-Chinese Wok Range-1-8 Holes.pdf</t>
         </is>
       </c>
+      <c r="G158" s="11" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n">
@@ -6956,6 +7180,7 @@
           <t>150 3-Burner Chinese Wok Range - Custom.pdf</t>
         </is>
       </c>
+      <c r="G159" s="11" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n">
@@ -6986,6 +7211,7 @@
           <t>149-149A-150-151-152_Imperial-Chinese Wok Range-1-8 Holes.pdf</t>
         </is>
       </c>
+      <c r="G160" s="11" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n">
@@ -7016,6 +7242,7 @@
           <t>151 FOUR BURNER CHINESE WOK RANGE.pdf</t>
         </is>
       </c>
+      <c r="G161" s="11" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n">
@@ -7046,6 +7273,7 @@
           <t>149-149A-150-151-152_Imperial-Chinese Wok Range-1-8 Holes.pdf</t>
         </is>
       </c>
+      <c r="G162" s="11" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n">
@@ -7076,6 +7304,7 @@
           <t>154_ IMPERIAL GRIDDLE_IMGA-2428-1.pdf</t>
         </is>
       </c>
+      <c r="G163" s="11" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n">
@@ -7106,6 +7335,7 @@
           <t>154 WELLS Countertop Griddle 2430G.pdf</t>
         </is>
       </c>
+      <c r="G164" s="11" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n">
@@ -7136,6 +7366,7 @@
           <t>155 WELLS 4 Burner2 2430G.pdf</t>
         </is>
       </c>
+      <c r="G165" s="11" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n">
@@ -7166,6 +7397,7 @@
           <t>156_Rinnai-Gas Rice Cooker_RER-55AS.pdf</t>
         </is>
       </c>
+      <c r="G166" s="11" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n">
@@ -7196,6 +7428,7 @@
           <t>157_Wells-Built-In Modular Warmers_300D-400D-500D.pdf</t>
         </is>
       </c>
+      <c r="G167" s="11" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n">
@@ -7226,6 +7459,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G168" s="11" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n">
@@ -7256,6 +7490,7 @@
           <t>161_Custom BBQ Chopping Table.pdf</t>
         </is>
       </c>
+      <c r="G169" s="11" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n">
@@ -7286,6 +7521,7 @@
           <t>162A Heated Display Cases HATC-GRHD.pdf</t>
         </is>
       </c>
+      <c r="G170" s="11" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n">
@@ -7316,6 +7552,7 @@
           <t>164_Zojirushi-Rice Warmer_THA-603.pdf</t>
         </is>
       </c>
+      <c r="G171" s="11" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n">
@@ -7346,6 +7583,7 @@
           <t>165_Amana Microwave RCS10DSE.pdf</t>
         </is>
       </c>
+      <c r="G172" s="11" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n">
@@ -7376,6 +7614,7 @@
           <t>166_Bunn-h5e-h5x1.pdf</t>
         </is>
       </c>
+      <c r="G173" s="11" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n">
@@ -7406,6 +7645,7 @@
           <t>L010 3-SIDE UPTURN EQUIPMENT STAND ES-ALLSS-24.pdf</t>
         </is>
       </c>
+      <c r="G174" s="11" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n">
@@ -7436,6 +7676,7 @@
           <t>172_ABS-Deck Oven Electric_ABSEDO283.pdf</t>
         </is>
       </c>
+      <c r="G175" s="11" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n">
@@ -7466,6 +7707,7 @@
           <t>174_Baxter-Single Wide Retarder Proofer_RPW1S.pdf</t>
         </is>
       </c>
+      <c r="G176" s="11" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n">
@@ -7496,6 +7738,7 @@
           <t>176_Oliver-Bread Slicer_797.pdf</t>
         </is>
       </c>
+      <c r="G177" s="11" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n">
@@ -7526,6 +7769,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G178" s="11" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n">
@@ -7556,6 +7800,7 @@
           <t>180_Globe-Bench Mixer 20 Qt_SP20.pdf</t>
         </is>
       </c>
+      <c r="G179" s="11" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n">
@@ -7586,6 +7831,7 @@
           <t>181_30QT Mixer_Hobart HL300.pdf</t>
         </is>
       </c>
+      <c r="G180" s="11" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n">
@@ -7616,6 +7862,7 @@
           <t>188 Island Hot Food Warmer Double Tier 3X6.pdf</t>
         </is>
       </c>
+      <c r="G181" s="11" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n">
@@ -7646,6 +7893,7 @@
           <t>189_Crathco-Premix Bev Dispenser_D25-4.pdf</t>
         </is>
       </c>
+      <c r="G182" s="11" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n">
@@ -7676,6 +7924,7 @@
           <t>190 Bunn Coffee Grinder 33700.0000.pdf</t>
         </is>
       </c>
+      <c r="G183" s="11" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n">
@@ -7706,6 +7955,7 @@
           <t>191 Bunn 27800.0009.pdf</t>
         </is>
       </c>
+      <c r="G184" s="11" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n">
@@ -7736,6 +7986,7 @@
           <t>195_Cup Sealing Machine.pdf</t>
         </is>
       </c>
+      <c r="G185" s="11" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n">
@@ -7766,6 +8017,7 @@
           <t>152_24 GRIDDLE BURNER AR-24G-2B.pdf</t>
         </is>
       </c>
+      <c r="G186" s="11" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n">
@@ -7796,6 +8048,7 @@
           <t>1-q82nfUD0KH-YMXZaRwonb95Yim2qfgE.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G187" s="11" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n">
@@ -7826,6 +8079,7 @@
           <t>198_MSF8303GR SANDWICH PREP TABLE.pdf</t>
         </is>
       </c>
+      <c r="G188" s="11" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n">
@@ -7856,6 +8110,7 @@
           <t>1q7gHl2HAskEG7exnZaJBJ8fRfgg-88go.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G189" s="11" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n">
@@ -7886,6 +8141,7 @@
           <t>145B_ ConvoTherm - C4 ET 20.20GB-N.SpecSheet.pdf</t>
         </is>
       </c>
+      <c r="G190" s="11" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n">
@@ -7916,6 +8172,7 @@
           <t>200_202 CNC MBF8505GR_MBF8507GR.pdf</t>
         </is>
       </c>
+      <c r="G191" s="11" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n">
@@ -7946,6 +8203,7 @@
           <t>201_203 CNC MBF8501GR_MBF8503GR.pdf</t>
         </is>
       </c>
+      <c r="G192" s="11" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n">
@@ -7976,6 +8234,7 @@
           <t>200_202 CNC MBF8505GR_MBF8507GR.pdf</t>
         </is>
       </c>
+      <c r="G193" s="11" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n">
@@ -8006,6 +8265,7 @@
           <t>201_203 CNC MBF8501GR_MBF8503GR.pdf</t>
         </is>
       </c>
+      <c r="G194" s="11" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n">
@@ -8036,6 +8296,7 @@
           <t>1gWFhPhwGzmd0ZcGWrO_u2iEcs_cEda_s.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G195" s="11" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n">
@@ -8066,6 +8327,7 @@
           <t>1e8tMZmRzbNLEB4IOUzOWpJNS4YGIH48q.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G196" s="11" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n">
@@ -8096,6 +8358,7 @@
           <t>1wzOQNjddjYtEjfiy2bOiR6k8HmDOLqyV.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G197" s="11" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n">
@@ -8126,6 +8389,7 @@
           <t>19UbalptlTxK9_ipFeTk0S5_nmBc0HJBM.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G198" s="11" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n">
@@ -8156,6 +8420,7 @@
           <t>1Un3Y9KV5bKbg88CK0NGlWrzfCf5Irw_o.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G199" s="11" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n">
@@ -8186,6 +8451,7 @@
           <t>1Qg2iNnGlgx7QycC7blcvjdzItjGMG3Dc.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G200" s="11" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n">
@@ -8216,6 +8482,7 @@
           <t>1EXKyyM2t0qnstmjh_51PkjM29iL-VswA.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G201" s="11" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n">
@@ -8246,6 +8513,7 @@
           <t>1TiNRJXD-BVF03pvpLTTJhJHbFD7dxBup.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G202" s="11" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n">
@@ -8276,6 +8544,7 @@
           <t>12aW94Yh_mVe6pSEry9E2EDJNL4KOVl0F.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G203" s="11" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n">
@@ -8306,6 +8575,7 @@
           <t>166_Bunn-h5e-h5x1.pdf</t>
         </is>
       </c>
+      <c r="G204" s="11" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n">
@@ -8336,6 +8606,7 @@
           <t>1TiNRJXD-BVF03pvpLTTJhJHbFD7dxBup.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G205" s="11" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n">
@@ -8366,6 +8637,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G206" s="11" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n">
@@ -8396,6 +8668,7 @@
           <t>L007 Double Stock Pot Stove ATSP-18-2L.pdf</t>
         </is>
       </c>
+      <c r="G207" s="11" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n">
@@ -8426,6 +8699,7 @@
           <t>1wS-5xoSOm2sSZNBrvOoW9xqjN8pmZcl-.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G208" s="11" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n">
@@ -8456,6 +8730,7 @@
           <t>061Hill Phoenix_i2i-Modular-Island-Case-Road-Map.pdf</t>
         </is>
       </c>
+      <c r="G209" s="11" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n">
@@ -8486,6 +8761,7 @@
           <t>见『待处理设备』表</t>
         </is>
       </c>
+      <c r="G210" s="11" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n">
@@ -8516,6 +8792,7 @@
           <t>117_General Equip-Service Counter-w-Sneeze Guard.pdf</t>
         </is>
       </c>
+      <c r="G211" s="11" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n">
@@ -8546,6 +8823,7 @@
           <t>1myNBxBTvWr6_bAyTj5_5nsRnjMGOeBCb.pdf（旧，建议抽查）</t>
         </is>
       </c>
+      <c r="G212" s="11" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n">
@@ -8576,12 +8854,18 @@
           <t>042_General Equip-Stainless Steel Front Service Counter.pdf</t>
         </is>
       </c>
+      <c r="G213" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="G5:G213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="设备状态" prompt="点单元格右侧箭头选择" type="list">
+      <formula1>"New,Existing,(E)Relocate,Remove"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>